<commit_message>
docs: add 3 missing frontend KPIs to P2P_KPIs.xlsx
- Leadership: SUMMARY_COUNTS (P2P Summary Counts panel — 10 JSON counters)
- Vendor: VENDOR_BREAKDOWN (Vendor Health Breakdown panel — JSON breakdown)
- Vendor: TOP_VENDOR_SPEND (Top-10 vendor spend chart — JSON array)

All 3 verified rendered in frontend via useKpi().find(); exact SQL from kpi_engine.py L1178/1271/1366.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/P2P_KPIs.xlsx
+++ b/P2P_KPIs.xlsx
@@ -263,7 +263,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -465,6 +465,45 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -831,7 +870,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H46"/>
+  <dimension ref="A1:H49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2361,6 +2400,111 @@
       <c r="G46" s="7" t="inlineStr">
         <is>
           <t>L1813</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="68" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="69" t="inlineStr">
+        <is>
+          <t>LEADERSHIP</t>
+        </is>
+      </c>
+      <c r="C47" s="70" t="inlineStr">
+        <is>
+          <t>SUMMARY_COUNTS</t>
+        </is>
+      </c>
+      <c r="D47" s="68" t="inlineStr">
+        <is>
+          <t>P2P Summary Counts (JSON)</t>
+        </is>
+      </c>
+      <c r="E47" s="68" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="F47" s="68" t="inlineStr">
+        <is>
+          <t>_leadership()</t>
+        </is>
+      </c>
+      <c r="G47" s="68" t="inlineStr">
+        <is>
+          <t>L1178</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="71" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="72" t="inlineStr">
+        <is>
+          <t>VENDOR</t>
+        </is>
+      </c>
+      <c r="C48" s="73" t="inlineStr">
+        <is>
+          <t>VENDOR_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="D48" s="71" t="inlineStr">
+        <is>
+          <t>Vendor Health Breakdown (JSON)</t>
+        </is>
+      </c>
+      <c r="E48" s="71" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="F48" s="71" t="inlineStr">
+        <is>
+          <t>_vendor()</t>
+        </is>
+      </c>
+      <c r="G48" s="71" t="inlineStr">
+        <is>
+          <t>L1271</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="68" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="74" t="inlineStr">
+        <is>
+          <t>VENDOR</t>
+        </is>
+      </c>
+      <c r="C49" s="70" t="inlineStr">
+        <is>
+          <t>TOP_VENDOR_SPEND</t>
+        </is>
+      </c>
+      <c r="D49" s="68" t="inlineStr">
+        <is>
+          <t>Top-10 Vendor Spend Share (JSON)</t>
+        </is>
+      </c>
+      <c r="E49" s="68" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="F49" s="68" t="inlineStr">
+        <is>
+          <t>_vendor()</t>
+        </is>
+      </c>
+      <c r="G49" s="68" t="inlineStr">
+        <is>
+          <t>L1366</t>
         </is>
       </c>
     </row>
@@ -3347,7 +3491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -3751,6 +3895,79 @@
         </is>
       </c>
     </row>
+    <row r="12" ht="300" customHeight="1">
+      <c r="A12" s="68" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="75" t="inlineStr">
+        <is>
+          <t>SUMMARY_COUNTS</t>
+        </is>
+      </c>
+      <c r="C12" s="68" t="inlineStr">
+        <is>
+          <t>P2P Summary Counts (JSON)</t>
+        </is>
+      </c>
+      <c r="D12" s="76" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="E12" s="23" t="inlineStr">
+        <is>
+          <t>JSON object with 10 pipeline counters rendered in the 'P2P Summary Counts' panel: approved_pr, approved_po, grn_lines, invoice_lines, payments (Pipeline Health); po_without_pr, one_time_vendors, po_no_contract, duplicate_invoices, sod_conflicts (Risk &amp; Exceptions). Stored in value_text; value_numeric is NULL.</t>
+        </is>
+      </c>
+      <c r="F12" s="24">
+        <f> JSON of 10 individual COUNT queries assembled in Python, stored as value_text</f>
+        <v/>
+      </c>
+      <c r="G12" s="25" t="inlineStr">
+        <is>
+          <t>-- 10 sub-queries assembled into JSON in Python (_leadership function):
+-- approved_pr
+SELECT COUNT(DISTINCT purchase_requisition || '|' || item_of_requisition)
+FROM pr_dump WHERE release_status IN ('X','XX','XXX','XXXX','XXXXX')
+-- approved_po
+SELECT COUNT(DISTINCT purchasing_document || '|' || item)
+FROM po_dump WHERE release_indicator = 'X' AND (deletion_indicator IS NULL OR deletion_indicator = '')
+-- grn_lines
+SELECT COUNT(*) FROM grn_dump WHERE debit_credit_ind = 'S'
+-- invoice_lines
+SELECT COUNT(*) FROM invoice_dump WHERE document_type IN ('RE','KR') AND CAST(amount_local_ccy AS REAL) &gt; 0
+-- payments
+SELECT COUNT(*) FROM payment_dump
+-- po_without_pr (Maverick POs)
+SELECT COUNT(DISTINCT purchasing_document) FROM po_dump
+WHERE (purchase_requisition IS NULL OR purchase_requisition = '')
+  AND (deletion_indicator IS NULL OR deletion_indicator = '')
+-- one_time_vendors
+SELECT COUNT(*) FROM vendor_master WHERE UPPER(vendor_type) = 'ONE_TIME'
+-- po_no_contract
+SELECT COUNT(*) FROM po_dump
+WHERE (contract_number IS NULL OR contract_number = '')
+  AND (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+-- duplicate_invoices (= DUPLICATE_INVOICE_COUNT l9)
+SELECT SUM(cnt - 1) FROM (
+    SELECT COUNT(DISTINCT invoice_doc) AS cnt FROM invoice_dump
+    WHERE document_type IN ('RE','KR')
+      AND (reverse_invoice IS NULL OR reverse_invoice = '')
+      AND invoice_doc NOT IN (
+          SELECT DISTINCT reverse_invoice FROM invoice_dump
+          WHERE reverse_invoice IS NOT NULL AND reverse_invoice != ''
+      )
+    GROUP BY company_code, vendor_invoice_ref, CAST(amount_local_ccy AS REAL), vendor, posting_date
+    HAVING COUNT(DISTINCT invoice_doc) &gt; 1
+)
+-- sod_conflicts (= SOD_CONFLICT_COUNT s7_total — sum of all 4 SOD types)
+-- see SOD_CONFLICT_COUNT row for full SQL
+-- JSON stored as: {"approved_pr":N,"approved_po":N,"grn_lines":N,"invoice_lines":N,
+--  "payments":N,"po_without_pr":N,"one_time_vendors":N,"po_no_contract":N,
+--  "duplicate_invoices":N,"sod_conflicts":N}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
@@ -3766,7 +3983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -4080,6 +4297,105 @@
 WHERE object_class = 'KRED'
   AND change_date &gt;= {MTD}
 -- object_class 'KRED' = SAP vendor master (LFB1/LFA1/LFM1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="228" customHeight="1">
+      <c r="A10" s="68" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="77" t="inlineStr">
+        <is>
+          <t>VENDOR_BREAKDOWN</t>
+        </is>
+      </c>
+      <c r="C10" s="68" t="inlineStr">
+        <is>
+          <t>Vendor Health Breakdown (JSON)</t>
+        </is>
+      </c>
+      <c r="D10" s="76" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="E10" s="23" t="inlineStr">
+        <is>
+          <t>JSON breakdown of vendor master data rendered in the 'Vendor Health Breakdown' section. Fields: active (3-block compliant), non_active (any block set), one_time, domestic, international, msme (msme_flag IN M/S), total, compliance_rate (%). 3-block compliance uses: central_purchasing_block, payment_block, posting_block_cc. value_numeric = compliance_rate; value_text = full JSON.</t>
+        </is>
+      </c>
+      <c r="F10" s="24">
+        <f> single SQL with 7 CASE/COUNT columns → assembled into JSON dict</f>
+        <v/>
+      </c>
+      <c r="G10" s="25" t="inlineStr">
+        <is>
+          <t>SELECT
+    COUNT(CASE WHEN (central_purchasing_block IS NULL OR central_purchasing_block &lt;&gt; 'X')
+                 AND (payment_block            IS NULL OR payment_block            &lt;&gt; '*')
+                 AND (posting_block_cc         IS NULL OR posting_block_cc         &lt;&gt; 'X')
+               THEN 1 END)                                        AS active,
+    COUNT(CASE WHEN central_purchasing_block = 'X'
+                  OR payment_block           = '*'
+                  OR posting_block_cc        = 'X'
+               THEN 1 END)                                        AS non_active,
+    COUNT(CASE WHEN UPPER(vendor_type) = 'ONE_TIME'      THEN 1 END) AS one_time,
+    COUNT(CASE WHEN UPPER(vendor_type) = 'DOMESTIC'      THEN 1 END) AS domestic,
+    COUNT(CASE WHEN UPPER(vendor_type) = 'INTERNATIONAL' THEN 1 END) AS international,
+    COUNT(CASE WHEN msme_flag IN ('M','S')               THEN 1 END) AS msme,
+    COUNT(*)                                                          AS total
+FROM vendor_master
+-- compliance_rate = active / total × 100 (computed in Python)
+-- JSON: {"active":N,"non_active":N,"one_time":N,"domestic":N,
+--         "international":N,"msme":N,"total":N,"compliance_rate":R}</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="204" customHeight="1">
+      <c r="A11" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="B11" s="79" t="inlineStr">
+        <is>
+          <t>TOP_VENDOR_SPEND</t>
+        </is>
+      </c>
+      <c r="C11" s="78" t="inlineStr">
+        <is>
+          <t>Top-10 Vendor Spend Share (JSON)</t>
+        </is>
+      </c>
+      <c r="D11" s="80" t="inlineStr">
+        <is>
+          <t>json</t>
+        </is>
+      </c>
+      <c r="E11" s="56" t="inlineStr">
+        <is>
+          <t>JSON array of top-10 vendors by total PO spend. Each entry: vendor (code), name, spend (INR), share_pct (% of total spend). Rendered as a bar/table chart in the Vendor dashboard. value_text only; value_numeric is NULL.</t>
+        </is>
+      </c>
+      <c r="F11" s="57">
+        <f> TOP 10 vendors by SUM(net_order_value); share_pct = vendor_spend / total_spend × 100</f>
+        <v/>
+      </c>
+      <c r="G11" s="58" t="inlineStr">
+        <is>
+          <t>-- Total spend (denominator)
+SELECT SUM(CAST(net_order_value AS REAL)) FROM po_dump
+WHERE (deletion_indicator IS NULL OR deletion_indicator NOT IN ('L','X'))
+-- Top-10 vendors
+SELECT po.vendor,
+       COALESCE(MIN(vm.vendor_name), MIN(po.vendor_name), po.vendor) AS name,
+       SUM(CAST(po.net_order_value AS REAL)) AS spend
+FROM po_dump po
+LEFT JOIN vendor_master vm ON po.vendor = vm.vendor
+WHERE (po.deletion_indicator IS NULL OR po.deletion_indicator NOT IN ('L','X'))
+GROUP BY po.vendor
+ORDER BY spend DESC
+LIMIT 10
+-- share_pct = spend / total_spend × 100 (computed in Python per row)
+-- JSON: [{"vendor":"V001","name":"ABC Ltd","spend":12345678.0,"share_pct":12.34}, ...]</t>
         </is>
       </c>
     </row>

</xml_diff>